<commit_message>
Sync latest douban movie collection workbook
</commit_message>
<xml_diff>
--- a/douban-movie-collector/examples/2026-09-04_电影资源收藏表.xlsx
+++ b/douban-movie-collector/examples/2026-09-04_电影资源收藏表.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="电影收藏" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'电影收藏'!$A$1:$R$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'电影收藏'!$A$1:$R$47</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'电影收藏'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -4234,74 +4234,362 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="n"/>
-      <c r="B43" s="3" t="n"/>
-      <c r="C43" s="2" t="n"/>
-      <c r="D43" s="4" t="n"/>
-      <c r="E43" s="2" t="n"/>
-      <c r="F43" s="3" t="n"/>
-      <c r="G43" s="8" t="n"/>
-      <c r="H43" s="2" t="n"/>
-      <c r="I43" s="9" t="n"/>
-      <c r="J43" s="7" t="n"/>
-      <c r="K43" s="2" t="n"/>
-      <c r="L43" s="3" t="n"/>
+      <c r="A43" s="31" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="32" t="inlineStr">
+        <is>
+          <t>电影</t>
+        </is>
+      </c>
+      <c r="C43" s="33" t="inlineStr">
+        <is>
+          <t>正发生</t>
+        </is>
+      </c>
+      <c r="D43" s="34" t="inlineStr">
+        <is>
+          <t>法国</t>
+        </is>
+      </c>
+      <c r="E43" s="46" t="n">
+        <v>2021</v>
+      </c>
+      <c r="F43" s="33" t="inlineStr">
+        <is>
+          <t>剧情</t>
+        </is>
+      </c>
+      <c r="G43" s="36" t="inlineStr">
+        <is>
+          <t>奥黛丽·迪万</t>
+        </is>
+      </c>
+      <c r="H43" s="47" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="I43" s="46" t="n"/>
+      <c r="J43" s="46" t="n"/>
+      <c r="K43" s="21" t="inlineStr">
+        <is>
+          <t>想看</t>
+        </is>
+      </c>
+      <c r="L43" s="48" t="n">
+        <v>46279</v>
+      </c>
+      <c r="M43" s="39" t="inlineStr">
+        <is>
+          <t>https://pan.quark.cn/s/01cc65fa1a7f</t>
+        </is>
+      </c>
+      <c r="N43" s="33" t="inlineStr">
+        <is>
+          <t>vEte</t>
+        </is>
+      </c>
+      <c r="O43" s="33" t="inlineStr">
+        <is>
+          <t>35318021</t>
+        </is>
+      </c>
+      <c r="P43" s="33" t="inlineStr">
+        <is>
+          <t>https://movie.douban.com/subject/35318021/</t>
+        </is>
+      </c>
+      <c r="Q43" s="48" t="n">
+        <v>46279</v>
+      </c>
+      <c r="R43" s="33" t="inlineStr">
+        <is>
+          <t>法国女大学生意外怀孕后，在法律限制与社会偏见中艰难寻求堕胎机会的剧情片，改编自安妮 埃尔诺自传作品。</t>
+        </is>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="n"/>
-      <c r="B44" s="3" t="n"/>
-      <c r="C44" s="2" t="n"/>
-      <c r="D44" s="4" t="n"/>
-      <c r="E44" s="2" t="n"/>
-      <c r="F44" s="3" t="n"/>
-      <c r="G44" s="8" t="n"/>
-      <c r="H44" s="2" t="n"/>
-      <c r="I44" s="9" t="n"/>
-      <c r="J44" s="7" t="n"/>
-      <c r="K44" s="2" t="n"/>
-      <c r="L44" s="3" t="n"/>
+      <c r="A44" s="31" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="32" t="inlineStr">
+        <is>
+          <t>电影</t>
+        </is>
+      </c>
+      <c r="C44" s="33" t="inlineStr">
+        <is>
+          <t>从不，很少，有时，总是</t>
+        </is>
+      </c>
+      <c r="D44" s="34" t="inlineStr">
+        <is>
+          <t>美国 / 英国</t>
+        </is>
+      </c>
+      <c r="E44" s="46" t="n">
+        <v>2020</v>
+      </c>
+      <c r="F44" s="33" t="inlineStr">
+        <is>
+          <t>剧情</t>
+        </is>
+      </c>
+      <c r="G44" s="36" t="inlineStr">
+        <is>
+          <t>伊丽莎·希特曼</t>
+        </is>
+      </c>
+      <c r="H44" s="47" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="I44" s="46" t="n"/>
+      <c r="J44" s="46" t="n"/>
+      <c r="K44" s="21" t="inlineStr">
+        <is>
+          <t>想看</t>
+        </is>
+      </c>
+      <c r="L44" s="48" t="n">
+        <v>46279</v>
+      </c>
+      <c r="M44" s="39" t="inlineStr">
+        <is>
+          <t>https://pan.quark.cn/s/1d4b4f9ecdb9</t>
+        </is>
+      </c>
+      <c r="N44" s="33" t="n"/>
+      <c r="O44" s="33" t="inlineStr">
+        <is>
+          <t>33411505</t>
+        </is>
+      </c>
+      <c r="P44" s="33" t="inlineStr">
+        <is>
+          <t>https://movie.douban.com/subject/33411505/</t>
+        </is>
+      </c>
+      <c r="Q44" s="48" t="n">
+        <v>46279</v>
+      </c>
+      <c r="R44" s="33" t="inlineStr">
+        <is>
+          <t>少女意外怀孕后，与表妹踏上前往纽约寻求堕胎帮助的旅程，影片以克制的镜头展现她们面对的困境与彼此扶持。</t>
+        </is>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="n"/>
-      <c r="B45" s="3" t="n"/>
-      <c r="C45" s="2" t="n"/>
-      <c r="D45" s="4" t="n"/>
-      <c r="E45" s="2" t="n"/>
-      <c r="F45" s="3" t="n"/>
-      <c r="G45" s="8" t="n"/>
-      <c r="H45" s="2" t="n"/>
-      <c r="I45" s="9" t="n"/>
-      <c r="J45" s="7" t="n"/>
-      <c r="K45" s="2" t="n"/>
-      <c r="L45" s="3" t="n"/>
+      <c r="A45" s="31" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="32" t="inlineStr">
+        <is>
+          <t>电影</t>
+        </is>
+      </c>
+      <c r="C45" s="33" t="inlineStr">
+        <is>
+          <t>毕业会考</t>
+        </is>
+      </c>
+      <c r="D45" s="34" t="inlineStr">
+        <is>
+          <t>罗马尼亚 / 法国 / 比利时</t>
+        </is>
+      </c>
+      <c r="E45" s="46" t="n">
+        <v>2016</v>
+      </c>
+      <c r="F45" s="33" t="inlineStr">
+        <is>
+          <t>剧情</t>
+        </is>
+      </c>
+      <c r="G45" s="36" t="inlineStr">
+        <is>
+          <t>克里斯蒂安·蒙吉</t>
+        </is>
+      </c>
+      <c r="H45" s="47" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="I45" s="46" t="n"/>
+      <c r="J45" s="46" t="n"/>
+      <c r="K45" s="21" t="inlineStr">
+        <is>
+          <t>想看</t>
+        </is>
+      </c>
+      <c r="L45" s="48" t="n">
+        <v>46279</v>
+      </c>
+      <c r="M45" s="39" t="inlineStr">
+        <is>
+          <t>https://pan.quark.cn/s/ddd53fcb40f0</t>
+        </is>
+      </c>
+      <c r="N45" s="33" t="n"/>
+      <c r="O45" s="33" t="inlineStr">
+        <is>
+          <t>26340305</t>
+        </is>
+      </c>
+      <c r="P45" s="33" t="inlineStr">
+        <is>
+          <t>https://movie.douban.com/subject/26340305/</t>
+        </is>
+      </c>
+      <c r="Q45" s="48" t="n">
+        <v>46279</v>
+      </c>
+      <c r="R45" s="33" t="inlineStr">
+        <is>
+          <t>女儿即将参加毕业会考，父亲却因一场意外被迫重新面对家庭、教育与人生选择，影片以克制笔触描绘东欧社会的现实困境。</t>
+        </is>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n"/>
-      <c r="B46" s="3" t="n"/>
-      <c r="C46" s="2" t="n"/>
-      <c r="D46" s="4" t="n"/>
-      <c r="E46" s="2" t="n"/>
-      <c r="F46" s="3" t="n"/>
-      <c r="G46" s="8" t="n"/>
-      <c r="H46" s="2" t="n"/>
-      <c r="I46" s="9" t="n"/>
-      <c r="J46" s="7" t="n"/>
-      <c r="K46" s="2" t="n"/>
-      <c r="L46" s="3" t="n"/>
+      <c r="A46" s="31" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="32" t="inlineStr">
+        <is>
+          <t>电影</t>
+        </is>
+      </c>
+      <c r="C46" s="33" t="inlineStr">
+        <is>
+          <t>和莎莫的500天</t>
+        </is>
+      </c>
+      <c r="D46" s="34" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="E46" s="46" t="n">
+        <v>2009</v>
+      </c>
+      <c r="F46" s="33" t="inlineStr">
+        <is>
+          <t>剧情 / 喜剧 / 爱情</t>
+        </is>
+      </c>
+      <c r="G46" s="36" t="inlineStr">
+        <is>
+          <t>马克·韦布</t>
+        </is>
+      </c>
+      <c r="H46" s="47" t="n">
+        <v>8</v>
+      </c>
+      <c r="I46" s="46" t="n"/>
+      <c r="J46" s="46" t="n"/>
+      <c r="K46" s="21" t="inlineStr">
+        <is>
+          <t>想看</t>
+        </is>
+      </c>
+      <c r="L46" s="48" t="n">
+        <v>46279</v>
+      </c>
+      <c r="M46" s="39" t="inlineStr">
+        <is>
+          <t>https://pan.quark.cn/s/86f962ca14f4</t>
+        </is>
+      </c>
+      <c r="N46" s="33" t="inlineStr">
+        <is>
+          <t>ufZ7</t>
+        </is>
+      </c>
+      <c r="O46" s="33" t="inlineStr">
+        <is>
+          <t>3072086</t>
+        </is>
+      </c>
+      <c r="P46" s="33" t="inlineStr">
+        <is>
+          <t>https://movie.douban.com/subject/3072086/</t>
+        </is>
+      </c>
+      <c r="Q46" s="48" t="n">
+        <v>46279</v>
+      </c>
+      <c r="R46" s="33" t="inlineStr">
+        <is>
+          <t>男孩汤姆遇见女孩莎莫，两人在一段充满甜蜜与错位的感情中彼此靠近又渐行渐远，回望这段恋情后重新认识爱与成长。</t>
+        </is>
+      </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="n"/>
-      <c r="B47" s="3" t="n"/>
-      <c r="C47" s="2" t="n"/>
-      <c r="D47" s="4" t="n"/>
-      <c r="E47" s="2" t="n"/>
-      <c r="F47" s="3" t="n"/>
-      <c r="G47" s="8" t="n"/>
-      <c r="H47" s="2" t="n"/>
-      <c r="I47" s="9" t="n"/>
-      <c r="J47" s="7" t="n"/>
-      <c r="K47" s="2" t="n"/>
-      <c r="L47" s="3" t="n"/>
+      <c r="A47" s="31" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="32" t="inlineStr">
+        <is>
+          <t>电影</t>
+        </is>
+      </c>
+      <c r="C47" s="33" t="inlineStr">
+        <is>
+          <t>春夏秋冬又一春</t>
+        </is>
+      </c>
+      <c r="D47" s="34" t="inlineStr">
+        <is>
+          <t>韩国 / 德国</t>
+        </is>
+      </c>
+      <c r="E47" s="46" t="n">
+        <v>2003</v>
+      </c>
+      <c r="F47" s="33" t="inlineStr">
+        <is>
+          <t>剧情</t>
+        </is>
+      </c>
+      <c r="G47" s="36" t="inlineStr">
+        <is>
+          <t>金基德</t>
+        </is>
+      </c>
+      <c r="H47" s="47" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="I47" s="46" t="n"/>
+      <c r="J47" s="46" t="n"/>
+      <c r="K47" s="21" t="inlineStr">
+        <is>
+          <t>想看</t>
+        </is>
+      </c>
+      <c r="L47" s="48" t="n">
+        <v>46279</v>
+      </c>
+      <c r="M47" s="39" t="inlineStr">
+        <is>
+          <t>https://pan.quark.cn/s/f71349ef40bb</t>
+        </is>
+      </c>
+      <c r="N47" s="33" t="n"/>
+      <c r="O47" s="33" t="inlineStr">
+        <is>
+          <t>1316580</t>
+        </is>
+      </c>
+      <c r="P47" s="33" t="inlineStr">
+        <is>
+          <t>https://movie.douban.com/subject/1316580/</t>
+        </is>
+      </c>
+      <c r="Q47" s="48" t="n">
+        <v>46279</v>
+      </c>
+      <c r="R47" s="33" t="inlineStr">
+        <is>
+          <t>湖上小寺中，男孩随师父修行成长，四季流转映照着欲望、罪责、救赎与人生轮回。</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n"/>
@@ -4486,7 +4774,7 @@
       <c r="L60" s="3" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R42"/>
+  <autoFilter ref="A1:R47"/>
   <conditionalFormatting sqref="H2:H60">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"已看"</formula>

</xml_diff>